<commit_message>
Source royalty-free assets from Pixabay/BBC with sourcing report
Add tools/source_assets.py to search Pixabay first (blocked by Cloudflare
in CI) then download from BBC Sound Effects archive. All 71 royalty-free
assets placed at expected paths with ffmpeg conversion. Generates
data/asset_sourcing_report.md and updates asset status/URLs.

Co-authored-by: perekl <perekl@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/master_sound_assets.xlsx
+++ b/data/master_sound_assets.xlsx
@@ -567,13 +567,17 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050196.wav</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Gail sessions, soft room tone.</t>
+          <t>Sourced from BBC Sound Effects — Primary School, classroom atmosphere in prefabricated building, 8-9 yo girls, some desk lids open &amp; closed, children mov</t>
         </is>
       </c>
     </row>
@@ -628,13 +632,17 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07070205.wav</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Sizzle, sidelines, ribs ready.</t>
+          <t xml:space="preserve">Sourced from BBC Sound Effects — Restaurant Kitchen atmosphere, with cooks chatting, food prepartion &amp; cooking sounds, extractor fan &amp; parking attendant </t>
         </is>
       </c>
     </row>
@@ -689,13 +697,17 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07026075.wav</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Counselor bunks, office phone scenes.</t>
+          <t>Sourced from BBC Sound Effects — Wooden Thames Sailing Barge: Cabin amidships, below deck underway in force 4 wind, interior</t>
         </is>
       </c>
     </row>
@@ -750,13 +762,17 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07030049.wav</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Hill, parking lot, bunk area, mess hall exterior, porches.</t>
+          <t>Sourced from BBC Sound Effects — Backgrounds: Atmosphere, Small Town, summer, birds, distant traffic and some speech. (Technical note, for use at low lev</t>
         </is>
       </c>
     </row>
@@ -811,13 +827,17 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050185.wav</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Field scramble, flagpole assembly murmur.</t>
+          <t>Sourced from BBC Sound Effects — Border Collies, exterior, about 10 months old, running around playing &amp; barking, with some early morning birdsong.</t>
         </is>
       </c>
     </row>
@@ -872,13 +892,17 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07024004.wav</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Fire crackle, crickets, night camp.</t>
+          <t>Sourced from BBC Sound Effects — Traction Engines (Single cylinder): Idling and fire burning, interior</t>
         </is>
       </c>
     </row>
@@ -933,13 +957,17 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07052029.wav</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Running, yelling, distant game.</t>
+          <t>Sourced from BBC Sound Effects — Greece: School playground, very noisy with children shouting &amp; playing, distant traffic, bell rings &amp; they go in.</t>
         </is>
       </c>
     </row>
@@ -994,13 +1022,17 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07006135.wav</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Ten years later gathering.</t>
+          <t>Sourced from BBC Sound Effects — Large crowd murmuring in a large room with echo.</t>
         </is>
       </c>
     </row>
@@ -1055,13 +1087,17 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050196.wav</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Crying, therapy, Gail breakdown support.</t>
+          <t>Sourced from BBC Sound Effects — Primary School, classroom atmosphere in prefabricated building, 8-9 yo girls, some desk lids open &amp; closed, children mov</t>
         </is>
       </c>
     </row>
@@ -1116,13 +1152,17 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068044.wav</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Van drive, lonely walk wind.</t>
+          <t>Sourced from BBC Sound Effects — Exterior - quiet cobbled side street off busy main road, wet weather, cars passing on cobbles.</t>
         </is>
       </c>
     </row>
@@ -1177,13 +1217,17 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07048070.wav</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Gene/Gary kitchen scenes.</t>
+          <t>Sourced from BBC Sound Effects — Temple dining room general atmosphere with chat (Hindi and English) and kitchen noise - good general-purpose background</t>
         </is>
       </c>
     </row>
@@ -1238,13 +1282,17 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034159.wav</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Swimming area, docks, lonely lake laps.</t>
+          <t>Sourced from BBC Sound Effects — English Electric Lightning, exterior, two waves of four planes passing over. (Jet engined fighter plane.)</t>
         </is>
       </c>
     </row>
@@ -1299,13 +1347,17 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07074036.wav</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Breakfast, dinner, tension, continue variants.</t>
+          <t>Sourced from BBC Sound Effects — American chatter; large mixed crowd in dining hall of US Air Force base.</t>
         </is>
       </c>
     </row>
@@ -1360,13 +1412,17 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07063011.wav</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Crickets, night work behind rec hall.</t>
+          <t>Sourced from BBC Sound Effects — British Saanen Goat, exterior, annoyed bleating, moving around a field (some close perspective calls), jackdaws &amp; cricke</t>
         </is>
       </c>
     </row>
@@ -1421,13 +1477,17 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07044130.wav</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Lake sunrise, garden morning, woods day, birds.</t>
+          <t>Sourced from BBC Sound Effects — Lake in early Spring,early morning atmosphere with Mallard, Coot, Canada Goose &amp; incipient dawn chorus, with Mallards ri</t>
         </is>
       </c>
     </row>
@@ -1482,13 +1542,17 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050206.wav</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Pre-show optional.</t>
+          <t>Sourced from BBC Sound Effects — School Computer Class, general atmosphere in pre-fabricated room, with hum from computers, keys clicking, occasional bac</t>
         </is>
       </c>
     </row>
@@ -1543,13 +1607,17 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07022535.wav</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Booth tone, static bed, broadcast under VO.</t>
+          <t>Sourced from BBC Sound Effects — Oil Rigs: Fortes Oilfield offshore rig. Atmosphere in radio room, fax receiver</t>
         </is>
       </c>
     </row>
@@ -1604,13 +1672,17 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07010033.wav</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Talent show rehearsal.</t>
+          <t>Sourced from BBC Sound Effects — Exterior, 2-tone into single-tone horn. (TR6 Sports Car, 1971 model)</t>
         </is>
       </c>
     </row>
@@ -1665,13 +1737,17 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07012124.wav</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Raft, danger rapids, Moose River.</t>
+          <t>Sourced from BBC Sound Effects — Rapids, rushing water. (Close perspective from river bank.)</t>
         </is>
       </c>
     </row>
@@ -1726,13 +1802,17 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07066144.wav</t>
+        </is>
+      </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Outdoor class, picnic table work.</t>
+          <t>Sourced from BBC Sound Effects — Airfield atmosphere - exterior (single engine jet fighter).</t>
         </is>
       </c>
     </row>
@@ -1787,13 +1867,17 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07028111.wav</t>
+        </is>
+      </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>JJ/Gary sneak scenes.</t>
+          <t>Sourced from BBC Sound Effects — Swimming: Pool atmosphere, water lapping, occasional splash, no swimmers</t>
         </is>
       </c>
     </row>
@@ -1848,13 +1932,17 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07057083.wav</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Rec hall murmur, settle, laughter bed.</t>
+          <t>Sourced from BBC Sound Effects — Audience in auditorium of provincial theatre (before perfomance)</t>
         </is>
       </c>
     </row>
@@ -1909,13 +1997,17 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07009124.wav</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Diegetic camper singing.</t>
+          <t>Sourced from BBC Sound Effects — Schoolchildren in classroom, mixed 10 to 13 year old pupils laughing. (Recorded in London, 1980.)</t>
         </is>
       </c>
     </row>
@@ -1970,13 +2062,17 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07024008.wav</t>
+        </is>
+      </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Victor/Neil hero run.</t>
+          <t>Sourced from BBC Sound Effects — Traction Engines (Single cylinder): Start, running, stop. Interior. Gear change at 1'25"</t>
         </is>
       </c>
     </row>
@@ -2031,13 +2127,17 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050174.wav</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Ben/McKinley wedding at forest lake.</t>
+          <t>Sourced from BBC Sound Effects — King Charles Spaniel, interior, scampering on wooden floor &amp; panting.</t>
         </is>
       </c>
     </row>
@@ -2092,13 +2192,17 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042202.wav</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Motorcycle chase.</t>
+          <t>Sourced from BBC Sound Effects — Single lamb bleating. (Comedy Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -2214,13 +2318,17 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Katie/Coop exterior reunion.</t>
+          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
         </is>
       </c>
     </row>
@@ -2275,13 +2383,17 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07020162.wav</t>
+        </is>
+      </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Optional post-show.</t>
+          <t>Sourced from BBC Sound Effects — London Underground station, atmosphere descending on escalator.</t>
         </is>
       </c>
     </row>
@@ -2336,13 +2448,17 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068065.wav</t>
+        </is>
+      </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Coop/Beth walk-off.</t>
+          <t>Sourced from BBC Sound Effects — Interior - Bucharest building site atmosphere, noisy with drills and hammering - close people in busy foyer acoustic.</t>
         </is>
       </c>
     </row>
@@ -2397,13 +2513,17 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07014173.wav</t>
+        </is>
+      </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Ten years later.</t>
+          <t>Sourced from BBC Sound Effects — Three harmonic stings. (Specially created electronic sound.)</t>
         </is>
       </c>
     </row>
@@ -2702,13 +2822,17 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032247.wav</t>
+        </is>
+      </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Coop/Gene training montage.</t>
+          <t>Sourced from BBC Sound Effects — Single rifles firing among rocks with ricochets. (Exterior recording.)</t>
         </is>
       </c>
     </row>
@@ -2763,13 +2887,17 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068065.wav</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Hill before dinner.</t>
+          <t>Sourced from BBC Sound Effects — Interior - Bucharest building site atmosphere, noisy with drills and hammering - close people in busy foyer acoustic.</t>
         </is>
       </c>
     </row>
@@ -2824,13 +2952,17 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07011152.wav</t>
+        </is>
+      </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Optional kiss moments.</t>
+          <t>Sourced from BBC Sound Effects — Exterior, door closed. (11.9 hp side valve Hotchkiss engine, 1922 Morris Bullnose.)</t>
         </is>
       </c>
     </row>
@@ -2885,13 +3017,17 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07004315.wav</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Capture the flag chase beat.</t>
+          <t>Sourced from BBC Sound Effects — Exterior, close start and depart. (Sports car, 1967 model)</t>
         </is>
       </c>
     </row>
@@ -3007,13 +3143,17 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>D20 die reveal.</t>
+          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
         </is>
       </c>
     </row>
@@ -3068,13 +3208,17 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07027076.wav</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Departure morning beats.</t>
+          <t>Sourced from BBC Sound Effects — Solid Panel Door: Interior, open and close. (Hall acoustic, close perspective)</t>
         </is>
       </c>
     </row>
@@ -3190,13 +3334,17 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043047.wav</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Light applause through standing ovation.</t>
+          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, crowd cheering.</t>
         </is>
       </c>
     </row>
@@ -3251,13 +3399,17 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043049.wav</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Post-Godspell reaction.</t>
+          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, boos and hisses.</t>
         </is>
       </c>
     </row>
@@ -3312,13 +3464,17 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043052.wav</t>
+        </is>
+      </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Talent show hysterics, group laughs.</t>
+          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, light laughter.</t>
         </is>
       </c>
     </row>
@@ -3373,13 +3529,17 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
+        </is>
+      </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Motorboat pass, ski boat.</t>
+          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
         </is>
       </c>
     </row>
@@ -3434,13 +3594,17 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034183.wav</t>
+        </is>
+      </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Thrown from van gags.</t>
+          <t>Sourced from BBC Sound Effects — Two body falls.</t>
         </is>
       </c>
     </row>
@@ -3495,13 +3659,17 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07045083.wav</t>
+        </is>
+      </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Silas departure, wagon leave.</t>
+          <t>Sourced from BBC Sound Effects — Railway Carriage, interior, door closed.</t>
         </is>
       </c>
     </row>
@@ -3556,13 +3724,17 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07005102.wav</t>
+        </is>
+      </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Urgent Skylab countdown optional.</t>
+          <t>Sourced from BBC Sound Effects — Atmosphere in a clock shop, with ticking and chimes. (Specially created effect)</t>
         </is>
       </c>
     </row>
@@ -3617,13 +3789,17 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
+        </is>
+      </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Crickets, rimshot, alien sting, shock stings.</t>
+          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -3678,13 +3854,17 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07022505.wav</t>
+        </is>
+      </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Plates, benches, door off hinges, Skylab.</t>
+          <t>Sourced from BBC Sound Effects — Crash: Window Breaking.</t>
         </is>
       </c>
     </row>
@@ -3739,13 +3919,17 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07065121.wav</t>
+        </is>
+      </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Van into tree.</t>
+          <t>Sourced from BBC Sound Effects — Car crash (no car noise) -1967 (84D)</t>
         </is>
       </c>
     </row>
@@ -3800,13 +3984,17 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043305.wav</t>
+        </is>
+      </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Skylab tracker sputter/power-up.</t>
+          <t>Sourced from BBC Sound Effects — High power phaser weapon., single shot. (Futuristic Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -3861,13 +4049,17 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043018.wav</t>
+        </is>
+      </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>D20 calibration scenes.</t>
+          <t>Sourced from BBC Sound Effects — Rolls Royce Silver Spirit, exterior, door opened &amp; closed. (6.75 litres, 1986 model.)</t>
         </is>
       </c>
     </row>
@@ -3922,13 +4114,17 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
+        </is>
+      </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Knock, creak, smash, infirmary bust-in.</t>
+          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
         </is>
       </c>
     </row>
@@ -3983,13 +4179,17 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07019171.wav</t>
+        </is>
+      </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Reveal, suspense, hero beats.</t>
+          <t>Sourced from BBC Sound Effects — Brown Bess Flintlock, single shot fired, hits metal target. (Manufactured 1757.)</t>
         </is>
       </c>
     </row>
@@ -4044,13 +4244,17 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
+        </is>
+      </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Van seat + Moose flamethrower layer.</t>
+          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -4105,13 +4309,17 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07003076.wav</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Screams, shouts, kid pile-on, wrestling.</t>
+          <t>Sourced from BBC Sound Effects — Children and clowns shout 'hello'. (Indistinguishable music in background)</t>
         </is>
       </c>
     </row>
@@ -4166,13 +4374,17 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032021.wav</t>
+        </is>
+      </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>Ring + mime ring in arts &amp; crafts.</t>
+          <t>Sourced from BBC Sound Effects — Leicester Tram, interior, passenger bell sounded, single rings. (Tram built 1904.)</t>
         </is>
       </c>
     </row>
@@ -4227,13 +4439,17 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07070120.wav</t>
+        </is>
+      </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>Paul traces call.</t>
+          <t>Sourced from BBC Sound Effects — Stromberg-Carlson - phone down.</t>
         </is>
       </c>
     </row>
@@ -4288,13 +4504,17 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07054042.wav</t>
+        </is>
+      </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Tray thud, tool clatter, mud squish, flag rope.</t>
+          <t>Sourced from BBC Sound Effects — Metallic impact crash (84F)</t>
         </is>
       </c>
     </row>
@@ -4349,13 +4569,17 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
+        </is>
+      </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Rec hall foundation shake.</t>
+          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
         </is>
       </c>
     </row>
@@ -4410,13 +4634,17 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07041190.wav</t>
+        </is>
+      </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Chases, bunk exits, night runs.</t>
+          <t>Sourced from BBC Sound Effects — Footsteps, two pairs of feet running away on gravel.</t>
         </is>
       </c>
     </row>
@@ -4471,13 +4699,17 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
+        </is>
+      </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Rake bonk, banana slip, bucket clunk.</t>
+          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -4532,13 +4764,17 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042169.wav</t>
+        </is>
+      </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Comedy smooch layers.</t>
+          <t>Sourced from BBC Sound Effects — Kiss. (Comedy Spot Effect.)</t>
         </is>
       </c>
     </row>
@@ -4593,13 +4829,17 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07005040.wav</t>
+        </is>
+      </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Cuts, dissolves, title cards, montage ticks.</t>
+          <t>Sourced from BBC Sound Effects — Whoosh bing bang doying. (Specially created effect)</t>
         </is>
       </c>
     </row>
@@ -4654,13 +4894,17 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032248.wav</t>
+        </is>
+      </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>BetaMax gag + epilogue projector.</t>
+          <t>Sourced from BBC Sound Effects — Old Hotel Lift, gates close, lift ascends &amp; stops, gates open. (No hum.)</t>
         </is>
       </c>
     </row>
@@ -4715,13 +4959,17 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07023055.wav</t>
+        </is>
+      </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>Tiger Claw arrival/departure.</t>
+          <t>Sourced from BBC Sound Effects — Cars: BMC car, 1000cc engine Interior, start, false starts, stop</t>
         </is>
       </c>
     </row>
@@ -4776,13 +5024,17 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L71" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050091.wav</t>
+        </is>
+      </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Approach, start, skid, night arrival.</t>
+          <t>Sourced from BBC Sound Effects — Land Rover, exterior, approach, pass &amp; depart. (Land Rover, Long Wheel Base, 109" Safari Diesel, Series 2A, 1967.)</t>
         </is>
       </c>
     </row>
@@ -4837,13 +5089,17 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
+        </is>
+      </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Beth's truck, door, peel-out.</t>
+          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
         </is>
       </c>
     </row>
@@ -4898,13 +5154,17 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
+        </is>
+      </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>Acceleration, doors, raft fall.</t>
+          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
         </is>
       </c>
     </row>
@@ -4959,13 +5219,17 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07009148.wav</t>
+        </is>
+      </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>DINNER, CAPTURE THE FLAG, kitchen yell.</t>
+          <t>Sourced from BBC Sound Effects — Marine Bugle Call, 'Officers dress for dinner'.</t>
         </is>
       </c>
     </row>
@@ -5020,13 +5284,17 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07038319.wav</t>
+        </is>
+      </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Lake fall, pool, ski drag.</t>
+          <t>Sourced from BBC Sound Effects — Splash in water.</t>
         </is>
       </c>
     </row>
@@ -5081,13 +5349,17 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034116.wav</t>
+        </is>
+      </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Capture flag, wolf whistles.</t>
+          <t>Sourced from BBC Sound Effects — Referee's whistle blown, single blast, double blast, long blast, longer blast.</t>
         </is>
       </c>
     </row>
@@ -5142,13 +5414,17 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/0009074.wav</t>
+        </is>
+      </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Steve power + Skylab redirect gust.</t>
+          <t>Sourced from BBC Sound Effects — weather - strong gusty wind</t>
         </is>
       </c>
     </row>
@@ -5203,13 +5479,17 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07045085.wav</t>
+        </is>
+      </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>Steve's initial breeze.</t>
+          <t>Sourced from BBC Sound Effects — Railway Carriage, interior, window closed (leather strap type).</t>
         </is>
       </c>
     </row>
@@ -5264,13 +5544,17 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr"/>
+          <t>Sourced</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>Reusable silence bed; cue duration/fade control behavior.</t>
+          <t>Sourced from generated</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Background Cue System v2 for live table-read operation
Introduce BACKGROUND vs FOREGROUND cue types with independent playback
channels. Background beds persist across foreground SFX/music; GO on
background cues fades and switches the bed without stopping foreground.

- tools/background_cues.py: classify cues and derive expected_background_asset_id
- master_cues.xlsx / cues.json: optional Cue Type and Expected Background Asset
- app/playback.py: dedicated background channel with pause, volume, elapsed
- app/soundboard.py: persistent Background panel, sync banner, mismatch dialog
- README: document operator-assist design (no automation)

Co-authored-by: perekl <perekl@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/master_sound_assets.xlsx
+++ b/data/master_sound_assets.xlsx
@@ -567,17 +567,13 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050196.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Primary School, classroom atmosphere in prefabricated building, 8-9 yo girls, some desk lids open &amp; closed, children mov</t>
+          <t>Gail sessions, soft room tone.</t>
         </is>
       </c>
     </row>
@@ -632,17 +628,13 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07070205.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sourced from BBC Sound Effects — Restaurant Kitchen atmosphere, with cooks chatting, food prepartion &amp; cooking sounds, extractor fan &amp; parking attendant </t>
+          <t>Sizzle, sidelines, ribs ready.</t>
         </is>
       </c>
     </row>
@@ -697,17 +689,13 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07026075.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Wooden Thames Sailing Barge: Cabin amidships, below deck underway in force 4 wind, interior</t>
+          <t>Counselor bunks, office phone scenes.</t>
         </is>
       </c>
     </row>
@@ -762,17 +750,13 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07030049.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Backgrounds: Atmosphere, Small Town, summer, birds, distant traffic and some speech. (Technical note, for use at low lev</t>
+          <t>Hill, parking lot, bunk area, mess hall exterior, porches.</t>
         </is>
       </c>
     </row>
@@ -827,17 +811,13 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050185.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Border Collies, exterior, about 10 months old, running around playing &amp; barking, with some early morning birdsong.</t>
+          <t>Field scramble, flagpole assembly murmur.</t>
         </is>
       </c>
     </row>
@@ -892,17 +872,13 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07024004.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Traction Engines (Single cylinder): Idling and fire burning, interior</t>
+          <t>Fire crackle, crickets, night camp.</t>
         </is>
       </c>
     </row>
@@ -957,17 +933,13 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07052029.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Greece: School playground, very noisy with children shouting &amp; playing, distant traffic, bell rings &amp; they go in.</t>
+          <t>Running, yelling, distant game.</t>
         </is>
       </c>
     </row>
@@ -1022,17 +994,13 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07006135.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Large crowd murmuring in a large room with echo.</t>
+          <t>Ten years later gathering.</t>
         </is>
       </c>
     </row>
@@ -1087,17 +1055,13 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050196.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Primary School, classroom atmosphere in prefabricated building, 8-9 yo girls, some desk lids open &amp; closed, children mov</t>
+          <t>Crying, therapy, Gail breakdown support.</t>
         </is>
       </c>
     </row>
@@ -1152,17 +1116,13 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068044.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Exterior - quiet cobbled side street off busy main road, wet weather, cars passing on cobbles.</t>
+          <t>Van drive, lonely walk wind.</t>
         </is>
       </c>
     </row>
@@ -1217,17 +1177,13 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07048070.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Temple dining room general atmosphere with chat (Hindi and English) and kitchen noise - good general-purpose background</t>
+          <t>Gene/Gary kitchen scenes.</t>
         </is>
       </c>
     </row>
@@ -1282,17 +1238,13 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034159.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — English Electric Lightning, exterior, two waves of four planes passing over. (Jet engined fighter plane.)</t>
+          <t>Swimming area, docks, lonely lake laps.</t>
         </is>
       </c>
     </row>
@@ -1347,17 +1299,13 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07074036.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — American chatter; large mixed crowd in dining hall of US Air Force base.</t>
+          <t>Breakfast, dinner, tension, continue variants.</t>
         </is>
       </c>
     </row>
@@ -1412,17 +1360,13 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07063011.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — British Saanen Goat, exterior, annoyed bleating, moving around a field (some close perspective calls), jackdaws &amp; cricke</t>
+          <t>Crickets, night work behind rec hall.</t>
         </is>
       </c>
     </row>
@@ -1477,17 +1421,13 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07044130.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Lake in early Spring,early morning atmosphere with Mallard, Coot, Canada Goose &amp; incipient dawn chorus, with Mallards ri</t>
+          <t>Lake sunrise, garden morning, woods day, birds.</t>
         </is>
       </c>
     </row>
@@ -1542,17 +1482,13 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050206.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — School Computer Class, general atmosphere in pre-fabricated room, with hum from computers, keys clicking, occasional bac</t>
+          <t>Pre-show optional.</t>
         </is>
       </c>
     </row>
@@ -1607,17 +1543,13 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07022535.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Oil Rigs: Fortes Oilfield offshore rig. Atmosphere in radio room, fax receiver</t>
+          <t>Booth tone, static bed, broadcast under VO.</t>
         </is>
       </c>
     </row>
@@ -1672,17 +1604,13 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07010033.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Exterior, 2-tone into single-tone horn. (TR6 Sports Car, 1971 model)</t>
+          <t>Talent show rehearsal.</t>
         </is>
       </c>
     </row>
@@ -1737,17 +1665,13 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07012124.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Rapids, rushing water. (Close perspective from river bank.)</t>
+          <t>Raft, danger rapids, Moose River.</t>
         </is>
       </c>
     </row>
@@ -1802,17 +1726,13 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07066144.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Airfield atmosphere - exterior (single engine jet fighter).</t>
+          <t>Outdoor class, picnic table work.</t>
         </is>
       </c>
     </row>
@@ -1867,17 +1787,13 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07028111.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Swimming: Pool atmosphere, water lapping, occasional splash, no swimmers</t>
+          <t>JJ/Gary sneak scenes.</t>
         </is>
       </c>
     </row>
@@ -1932,17 +1848,13 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07057083.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Audience in auditorium of provincial theatre (before perfomance)</t>
+          <t>Rec hall murmur, settle, laughter bed.</t>
         </is>
       </c>
     </row>
@@ -1997,17 +1909,13 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07009124.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Schoolchildren in classroom, mixed 10 to 13 year old pupils laughing. (Recorded in London, 1980.)</t>
+          <t>Diegetic camper singing.</t>
         </is>
       </c>
     </row>
@@ -2062,17 +1970,13 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07024008.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Traction Engines (Single cylinder): Start, running, stop. Interior. Gear change at 1'25"</t>
+          <t>Victor/Neil hero run.</t>
         </is>
       </c>
     </row>
@@ -2127,17 +2031,13 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050174.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — King Charles Spaniel, interior, scampering on wooden floor &amp; panting.</t>
+          <t>Ben/McKinley wedding at forest lake.</t>
         </is>
       </c>
     </row>
@@ -2192,17 +2092,13 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042202.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Single lamb bleating. (Comedy Spot Effect.)</t>
+          <t>Motorcycle chase.</t>
         </is>
       </c>
     </row>
@@ -2318,17 +2214,13 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
+          <t>Katie/Coop exterior reunion.</t>
         </is>
       </c>
     </row>
@@ -2383,17 +2275,13 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07020162.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — London Underground station, atmosphere descending on escalator.</t>
+          <t>Optional post-show.</t>
         </is>
       </c>
     </row>
@@ -2448,17 +2336,13 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068065.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Interior - Bucharest building site atmosphere, noisy with drills and hammering - close people in busy foyer acoustic.</t>
+          <t>Coop/Beth walk-off.</t>
         </is>
       </c>
     </row>
@@ -2513,17 +2397,13 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07014173.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Three harmonic stings. (Specially created electronic sound.)</t>
+          <t>Ten years later.</t>
         </is>
       </c>
     </row>
@@ -2822,17 +2702,13 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032247.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Single rifles firing among rocks with ricochets. (Exterior recording.)</t>
+          <t>Coop/Gene training montage.</t>
         </is>
       </c>
     </row>
@@ -2887,17 +2763,13 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07068065.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Interior - Bucharest building site atmosphere, noisy with drills and hammering - close people in busy foyer acoustic.</t>
+          <t>Hill before dinner.</t>
         </is>
       </c>
     </row>
@@ -2952,17 +2824,13 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07011152.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Exterior, door closed. (11.9 hp side valve Hotchkiss engine, 1922 Morris Bullnose.)</t>
+          <t>Optional kiss moments.</t>
         </is>
       </c>
     </row>
@@ -3017,17 +2885,13 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07004315.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Exterior, close start and depart. (Sports car, 1967 model)</t>
+          <t>Capture the flag chase beat.</t>
         </is>
       </c>
     </row>
@@ -3143,17 +3007,13 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
+          <t>D20 die reveal.</t>
         </is>
       </c>
     </row>
@@ -3208,17 +3068,13 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07027076.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Solid Panel Door: Interior, open and close. (Hall acoustic, close perspective)</t>
+          <t>Departure morning beats.</t>
         </is>
       </c>
     </row>
@@ -3334,17 +3190,13 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043047.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, crowd cheering.</t>
+          <t>Light applause through standing ovation.</t>
         </is>
       </c>
     </row>
@@ -3399,17 +3251,13 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043049.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, boos and hisses.</t>
+          <t>Post-Godspell reaction.</t>
         </is>
       </c>
     </row>
@@ -3464,17 +3312,13 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043052.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Light Entertainment Audience, light laughter.</t>
+          <t>Talent show hysterics, group laughs.</t>
         </is>
       </c>
     </row>
@@ -3529,17 +3373,13 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
+          <t>Motorboat pass, ski boat.</t>
         </is>
       </c>
     </row>
@@ -3594,17 +3434,13 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034183.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Two body falls.</t>
+          <t>Thrown from van gags.</t>
         </is>
       </c>
     </row>
@@ -3659,17 +3495,13 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07045083.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Railway Carriage, interior, door closed.</t>
+          <t>Silas departure, wagon leave.</t>
         </is>
       </c>
     </row>
@@ -3724,17 +3556,13 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07005102.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Atmosphere in a clock shop, with ticking and chimes. (Specially created effect)</t>
+          <t>Urgent Skylab countdown optional.</t>
         </is>
       </c>
     </row>
@@ -3789,17 +3617,13 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
+          <t>Crickets, rimshot, alien sting, shock stings.</t>
         </is>
       </c>
     </row>
@@ -3854,17 +3678,13 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07022505.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Crash: Window Breaking.</t>
+          <t>Plates, benches, door off hinges, Skylab.</t>
         </is>
       </c>
     </row>
@@ -3919,17 +3739,13 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07065121.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Car crash (no car noise) -1967 (84D)</t>
+          <t>Van into tree.</t>
         </is>
       </c>
     </row>
@@ -3984,17 +3800,13 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043305.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — High power phaser weapon., single shot. (Futuristic Spot Effect.)</t>
+          <t>Skylab tracker sputter/power-up.</t>
         </is>
       </c>
     </row>
@@ -4049,17 +3861,13 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07043018.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Rolls Royce Silver Spirit, exterior, door opened &amp; closed. (6.75 litres, 1986 model.)</t>
+          <t>D20 calibration scenes.</t>
         </is>
       </c>
     </row>
@@ -4114,17 +3922,13 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
+          <t>Knock, creak, smash, infirmary bust-in.</t>
         </is>
       </c>
     </row>
@@ -4179,17 +3983,13 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07019171.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Brown Bess Flintlock, single shot fired, hits metal target. (Manufactured 1757.)</t>
+          <t>Reveal, suspense, hero beats.</t>
         </is>
       </c>
     </row>
@@ -4244,17 +4044,13 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
+          <t>Van seat + Moose flamethrower layer.</t>
         </is>
       </c>
     </row>
@@ -4309,17 +4105,13 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07003076.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Children and clowns shout 'hello'. (Indistinguishable music in background)</t>
+          <t>Screams, shouts, kid pile-on, wrestling.</t>
         </is>
       </c>
     </row>
@@ -4374,17 +4166,13 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032021.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Leicester Tram, interior, passenger bell sounded, single rings. (Tram built 1904.)</t>
+          <t>Ring + mime ring in arts &amp; crafts.</t>
         </is>
       </c>
     </row>
@@ -4439,17 +4227,13 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07070120.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Stromberg-Carlson - phone down.</t>
+          <t>Paul traces call.</t>
         </is>
       </c>
     </row>
@@ -4504,17 +4288,13 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07054042.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Metallic impact crash (84F)</t>
+          <t>Tray thud, tool clatter, mud squish, flag rope.</t>
         </is>
       </c>
     </row>
@@ -4569,17 +4349,13 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07055152.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — exterior - single bleep rec. from close perspective, as for arming</t>
+          <t>Rec hall foundation shake.</t>
         </is>
       </c>
     </row>
@@ -4634,17 +4410,13 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07041190.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Footsteps, two pairs of feet running away on gravel.</t>
+          <t>Chases, bunk exits, night runs.</t>
         </is>
       </c>
     </row>
@@ -4699,17 +4471,13 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042162.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Single burp. (Comedy Spot Effect.)</t>
+          <t>Rake bonk, banana slip, bucket clunk.</t>
         </is>
       </c>
     </row>
@@ -4764,17 +4532,13 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07042169.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Kiss. (Comedy Spot Effect.)</t>
+          <t>Comedy smooch layers.</t>
         </is>
       </c>
     </row>
@@ -4829,17 +4593,13 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07005040.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Whoosh bing bang doying. (Specially created effect)</t>
+          <t>Cuts, dissolves, title cards, montage ticks.</t>
         </is>
       </c>
     </row>
@@ -4894,17 +4654,13 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07032248.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr"/>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Old Hotel Lift, gates close, lift ascends &amp; stops, gates open. (No hum.)</t>
+          <t>BetaMax gag + epilogue projector.</t>
         </is>
       </c>
     </row>
@@ -4959,17 +4715,13 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07023055.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr"/>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Cars: BMC car, 1000cc engine Interior, start, false starts, stop</t>
+          <t>Tiger Claw arrival/departure.</t>
         </is>
       </c>
     </row>
@@ -5024,17 +4776,13 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07050091.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr"/>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Land Rover, exterior, approach, pass &amp; depart. (Land Rover, Long Wheel Base, 109" Safari Diesel, Series 2A, 1967.)</t>
+          <t>Approach, start, skid, night arrival.</t>
         </is>
       </c>
     </row>
@@ -5089,17 +4837,13 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
+          <t>Beth's truck, door, peel-out.</t>
         </is>
       </c>
     </row>
@@ -5154,17 +4898,13 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07051123.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Cessna C150, exterior, door opened &amp; closed. (Light aircraft, single piston engine.)</t>
+          <t>Acceleration, doors, raft fall.</t>
         </is>
       </c>
     </row>
@@ -5219,17 +4959,13 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07009148.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Marine Bugle Call, 'Officers dress for dinner'.</t>
+          <t>DINNER, CAPTURE THE FLAG, kitchen yell.</t>
         </is>
       </c>
     </row>
@@ -5284,17 +5020,13 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07038319.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Splash in water.</t>
+          <t>Lake fall, pool, ski drag.</t>
         </is>
       </c>
     </row>
@@ -5349,17 +5081,13 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07034116.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Referee's whistle blown, single blast, double blast, long blast, longer blast.</t>
+          <t>Capture flag, wolf whistles.</t>
         </is>
       </c>
     </row>
@@ -5414,17 +5142,13 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/0009074.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — weather - strong gusty wind</t>
+          <t>Steve power + Skylab redirect gust.</t>
         </is>
       </c>
     </row>
@@ -5479,17 +5203,13 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>https://sound-effects-media.bbcrewind.co.uk/wav/07045085.wav</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>Sourced from BBC Sound Effects — Railway Carriage, interior, window closed (leather strap type).</t>
+          <t>Steve's initial breeze.</t>
         </is>
       </c>
     </row>
@@ -5544,17 +5264,13 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>Sourced</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr">
-        <is>
-          <t>generated</t>
-        </is>
-      </c>
+          <t>Needed</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr"/>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>Sourced from generated</t>
+          <t>Reusable silence bed; cue duration/fade control behavior.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fresh cue placements: songs as background, improved line matching
- Reclassify all Music cues as Ambience (BACKGROUND); remove MUSIC UI category
- Clear and regenerate script.json placements from scratch via import heuristics
- Improve placement scoring: trigger phrase match beats scene-heading fallback
- Remove legacy Music playback branch; update README marker docs

Co-authored-by: perekl <perekl@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/master_sound_assets.xlsx
+++ b/data/master_sound_assets.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>CUE-005, CUE-034, CUE-035, CUE-045, CUE-203, CUE-051, CUE-205, CUE-063, CUE-066, CUE-085, CUE-090, CUE-213, CUE-215, CUE-216, CUE-217, CUE-117, CUE-156, CUE-184, CUE-188</t>
+          <t>CUE-005, CUE-034, CUE-035, CUE-045, CUE-203, CUE-051, CUE-205, CUE-063, CUE-066, CUE-085, CUE-090, CUE-213, CUE-215, CUE-216, CUE-217, CUE-117, CUE-221, CUE-156, CUE-181, CUE-184, CUE-188</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1871,16 +1871,16 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1932,16 +1932,16 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1993,16 +1993,16 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -2054,16 +2054,16 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -2115,16 +2115,16 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -2176,16 +2176,16 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -2237,16 +2237,16 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2298,16 +2298,16 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2359,16 +2359,16 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2420,16 +2420,16 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2481,16 +2481,16 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2542,16 +2542,16 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2664,16 +2664,16 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2776,26 +2776,26 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AST-039</t>
+          <t>AST-040</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Romantic Kiss Stinger</t>
+          <t>Slo-Mo Sports Underscore</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2809,17 +2809,17 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_romantic_kiss_stinger.mp3</t>
+          <t>assets/generated/music_slo_mo_sports.mp3</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>4s</t>
+          <t>30s</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>CUE-221, CUE-181</t>
+          <t>CUE-099</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -2830,57 +2830,57 @@
       <c r="L39" s="2" t="inlineStr"/>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Optional kiss moments.</t>
+          <t>Capture the flag chase beat.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AST-040</t>
+          <t>AST-041</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Slo-Mo Sports Underscore</t>
+          <t>Summer in the City (Lovin' Spoonful)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Royalty-free</t>
+          <t>Licensed - Lovin' Spoonful</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_slo_mo_sports.mp3</t>
+          <t>assets/generated/music_summer_in_the_city.mp3</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>30s</t>
+          <t>Full/skip</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>CUE-099</t>
+          <t>CUE-116</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -2891,57 +2891,57 @@
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>Capture the flag chase beat.</t>
+          <t>Arty radio into mess hall exteriors.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AST-041</t>
+          <t>AST-042</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Summer in the City (Lovin' Spoonful)</t>
+          <t>Symphonic Hope Crescendo</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Licensed - Lovin' Spoonful</t>
+          <t>Royalty-free orchestral</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_summer_in_the_city.mp3</t>
+          <t>assets/generated/music_symphonic_hope_crescendo.mp3</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Full/skip</t>
+          <t>8s</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>CUE-116</t>
+          <t>CUE-154</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2952,33 +2952,33 @@
       <c r="L41" s="2" t="inlineStr"/>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Arty radio into mess hall exteriors.</t>
+          <t>D20 die reveal.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AST-042</t>
+          <t>AST-043</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Symphonic Hope Crescendo</t>
+          <t>Warm Morning Sting</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2987,22 +2987,22 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Royalty-free orchestral</t>
+          <t>Royalty-free</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_symphonic_hope_crescendo.mp3</t>
+          <t>assets/generated/music_warm_morning_sting.mp3</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>8s</t>
+          <t>5s</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>CUE-154</t>
+          <t>CUE-237</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3013,57 +3013,57 @@
       <c r="L42" s="2" t="inlineStr"/>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>D20 die reveal.</t>
+          <t>Departure morning beats.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AST-043</t>
+          <t>AST-044</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Warm Morning Sting</t>
+          <t>You've Got a Friend (Campers)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Ambience</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Royalty-free</t>
+          <t>Licensed - Carole King</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_warm_morning_sting.mp3</t>
+          <t>assets/generated/music_youve_got_a_friend_campers.mp3</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>5s</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>CUE-237</t>
+          <t>CUE-157</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3074,57 +3074,57 @@
       <c r="L43" s="2" t="inlineStr"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Departure morning beats.</t>
+          <t>Bunk 7 talent show act.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AST-044</t>
+          <t>AST-045</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>You've Got a Friend (Campers)</t>
+          <t>Applause / Cheer</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>SFX</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Music</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Licensed - Carole King</t>
+          <t>Freesound</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>assets/generated/music_youve_got_a_friend_campers.mp3</t>
+          <t>assets/sfx/applause_cheer.wav</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>3-15s</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>CUE-157</t>
+          <t>CUE-049, CUE-064, CUE-106, CUE-113, CUE-120, CUE-121, CUE-124, CUE-151, CUE-160, CUE-162, CUE-164, CUE-166, CUE-180</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3135,19 +3135,19 @@
       <c r="L44" s="2" t="inlineStr"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Bunk 7 talent show act.</t>
+          <t>Light applause through standing ovation.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AST-045</t>
+          <t>AST-046</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Applause / Cheer</t>
+          <t>Audience Boo / Hiss</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3175,17 +3175,17 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/applause_cheer.wav</t>
+          <t>assets/sfx/audience_boo_hiss.wav</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>3-15s</t>
+          <t>6s</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>CUE-049, CUE-064, CUE-106, CUE-113, CUE-120, CUE-121, CUE-124, CUE-151, CUE-160, CUE-162, CUE-164, CUE-166, CUE-180</t>
+          <t>CUE-167</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3196,19 +3196,19 @@
       <c r="L45" s="2" t="inlineStr"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Light applause through standing ovation.</t>
+          <t>Post-Godspell reaction.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AST-046</t>
+          <t>AST-047</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Audience Boo / Hiss</t>
+          <t>Audience Laughter</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3236,17 +3236,17 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/audience_boo_hiss.wav</t>
+          <t>assets/sfx/audience_laughter.wav</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>6s</t>
+          <t>4-8s</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>CUE-167</t>
+          <t>CUE-067, CUE-159, CUE-185</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3257,19 +3257,19 @@
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Post-Godspell reaction.</t>
+          <t>Talent show hysterics, group laughs.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AST-047</t>
+          <t>AST-050</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Audience Laughter</t>
+          <t>Boat Engine</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3297,17 +3297,17 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/audience_laughter.wav</t>
+          <t>assets/sfx/boat_engine.wav</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>4-8s</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>CUE-067, CUE-159, CUE-185</t>
+          <t>CUE-053, CUE-218</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3318,19 +3318,19 @@
       <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Talent show hysterics, group laughs.</t>
+          <t>Motorboat pass, ski boat.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>AST-050</t>
+          <t>AST-051</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Boat Engine</t>
+          <t>Body Tumble / Roll</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3358,17 +3358,17 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/boat_engine.wav</t>
+          <t>assets/sfx/body_tumble_roll.wav</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>3s</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>CUE-053, CUE-218</t>
+          <t>CUE-060, CUE-101</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -3379,19 +3379,19 @@
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Motorboat pass, ski boat.</t>
+          <t>Thrown from van gags.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>AST-051</t>
+          <t>AST-053</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Body Tumble / Roll</t>
+          <t>Car Door</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3419,17 +3419,17 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/body_tumble_roll.wav</t>
+          <t>assets/sfx/car_door.wav</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>3s</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>CUE-060, CUE-101</t>
+          <t>CUE-189</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -3440,33 +3440,33 @@
       <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Thrown from van gags.</t>
+          <t>Silas departure, wagon leave.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>AST-053</t>
+          <t>AST-054</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Car Door</t>
+          <t>Clock Tick (Optional)</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>SFX</t>
+          <t>Comedy</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3480,17 +3480,17 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/car_door.wav</t>
+          <t>assets/sfx/clock_tick_optional.wav</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>CUE-189</t>
+          <t>CUE-234</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -3501,19 +3501,19 @@
       <c r="L50" s="2" t="inlineStr"/>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Silas departure, wagon leave.</t>
+          <t>Urgent Skylab countdown optional.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>AST-054</t>
+          <t>AST-055</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Clock Tick (Optional)</t>
+          <t>Comedy Stinger</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -3523,11 +3523,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3541,17 +3541,17 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/clock_tick_optional.wav</t>
+          <t>assets/sfx/comedy_stinger.wav</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>1-3s</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>CUE-234</t>
+          <t>CUE-030, CUE-212, CUE-103, CUE-228, CUE-150, CUE-231, CUE-238</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -3562,24 +3562,24 @@
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Urgent Skylab countdown optional.</t>
+          <t>Crickets, rimshot, alien sting, shock stings.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>AST-055</t>
+          <t>AST-056</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Comedy Stinger</t>
+          <t>Impact / Crash Debris</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Comedy</t>
+          <t>SFX</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -3602,17 +3602,17 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/comedy_stinger.wav</t>
+          <t>assets/sfx/crash_impact_debris.wav</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>1-3s</t>
+          <t>3s</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>CUE-030, CUE-212, CUE-103, CUE-228, CUE-150, CUE-231, CUE-238</t>
+          <t>CUE-047, CUE-119, CUE-175, CUE-178, CUE-182</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -3623,19 +3623,19 @@
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Crickets, rimshot, alien sting, shock stings.</t>
+          <t>Plates, benches, door off hinges, Skylab.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>AST-056</t>
+          <t>AST-057</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Impact / Crash Debris</t>
+          <t>Vehicle Crash</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3663,17 +3663,17 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/crash_impact_debris.wav</t>
+          <t>assets/sfx/crash_vehicle.wav</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>3s</t>
+          <t>4s</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>CUE-047, CUE-119, CUE-175, CUE-178, CUE-182</t>
+          <t>CUE-074</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -3684,19 +3684,19 @@
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Plates, benches, door off hinges, Skylab.</t>
+          <t>Van into tree.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>AST-057</t>
+          <t>AST-059</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Vehicle Crash</t>
+          <t>Sci-Fi Device</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/crash_vehicle.wav</t>
+          <t>assets/sfx/scifi_device.wav</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>CUE-074</t>
+          <t>CUE-145, CUE-176</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -3745,19 +3745,19 @@
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Van into tree.</t>
+          <t>Skylab tracker sputter/power-up.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>AST-059</t>
+          <t>AST-060</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Sci-Fi Device</t>
+          <t>Dice Roll</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/scifi_device.wav</t>
+          <t>assets/sfx/dice_roll.wav</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>4s</t>
+          <t>1s</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>CUE-145, CUE-176</t>
+          <t>CUE-153, CUE-158, CUE-168</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -3806,19 +3806,19 @@
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Skylab tracker sputter/power-up.</t>
+          <t>D20 calibration scenes.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>AST-060</t>
+          <t>AST-061</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Dice Roll</t>
+          <t>Door</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3846,17 +3846,17 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/dice_roll.wav</t>
+          <t>assets/sfx/door.wav</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>1s</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>CUE-153, CUE-158, CUE-168</t>
+          <t>CUE-037, CUE-072, CUE-211, CUE-112, CUE-140, CUE-170</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -3867,24 +3867,24 @@
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>D20 calibration scenes.</t>
+          <t>Knock, creak, smash, infirmary bust-in.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>AST-061</t>
+          <t>AST-062</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Door</t>
+          <t>Dramatic Stinger</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>SFX</t>
+          <t>Transition</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/door.wav</t>
+          <t>assets/sfx/dramatic_stinger.wav</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3917,7 +3917,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>CUE-037, CUE-072, CUE-211, CUE-112, CUE-140, CUE-170</t>
+          <t>CUE-227, CUE-147, CUE-152, CUE-163</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -3928,24 +3928,24 @@
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Knock, creak, smash, infirmary bust-in.</t>
+          <t>Reveal, suspense, hero beats.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>AST-062</t>
+          <t>AST-063</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Dramatic Stinger</t>
+          <t>Comedy Fart</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Transition</t>
+          <t>SFX</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/dramatic_stinger.wav</t>
+          <t>assets/sfx/comedy_fart.wav</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>CUE-227, CUE-147, CUE-152, CUE-163</t>
+          <t>CUE-161</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -3989,19 +3989,19 @@
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Reveal, suspense, hero beats.</t>
+          <t>Van seat + Moose flamethrower layer.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>AST-063</t>
+          <t>AST-064</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Comedy Fart</t>
+          <t>Human Reaction</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4024,22 +4024,22 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Freesound</t>
+          <t>Freesound / live</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/comedy_fart.wav</t>
+          <t>assets/sfx/human_reaction.wav</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>2-5s</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>CUE-161</t>
+          <t>CUE-016, CUE-038, CUE-040, CUE-110, CUE-122, CUE-123</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -4050,19 +4050,19 @@
       <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>Van seat + Moose flamethrower layer.</t>
+          <t>Screams, shouts, kid pile-on, wrestling.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>AST-064</t>
+          <t>AST-066</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Human Reaction</t>
+          <t>Telephone</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4085,22 +4085,22 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Freesound / live</t>
+          <t>Freesound</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/human_reaction.wav</t>
+          <t>assets/sfx/telephone_ring.wav</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>2-5s</t>
+          <t>3s</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>CUE-016, CUE-038, CUE-040, CUE-110, CUE-122, CUE-123</t>
+          <t>CUE-044, CUE-105, CUE-138</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -4111,19 +4111,19 @@
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>Screams, shouts, kid pile-on, wrestling.</t>
+          <t>Ring + mime ring in arts &amp; crafts.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>AST-066</t>
+          <t>AST-067</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Telephone</t>
+          <t>Phone Trace Beeps</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4151,17 +4151,17 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/telephone_ring.wav</t>
+          <t>assets/sfx/phone_trace_beeps.wav</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>3s</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>CUE-044, CUE-105, CUE-138</t>
+          <t>CUE-139</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -4172,19 +4172,19 @@
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>Ring + mime ring in arts &amp; crafts.</t>
+          <t>Paul traces call.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AST-067</t>
+          <t>AST-068</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Phone Trace Beeps</t>
+          <t>Prop Impact</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4212,17 +4212,17 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/phone_trace_beeps.wav</t>
+          <t>assets/sfx/prop_impact.wav</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>CUE-139</t>
+          <t>CUE-011, CUE-017, CUE-020, CUE-024, CUE-025, CUE-031, CUE-058, CUE-095, CUE-226</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -4233,19 +4233,19 @@
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>Paul traces call.</t>
+          <t>Tray thud, tool clatter, mud squish, flag rope.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AST-068</t>
+          <t>AST-069</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Prop Impact</t>
+          <t>Rumble / Building Shake</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -4273,17 +4273,17 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/prop_impact.wav</t>
+          <t>assets/sfx/rumble_building_shake.wav</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>6s</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>CUE-011, CUE-017, CUE-020, CUE-024, CUE-025, CUE-031, CUE-058, CUE-095, CUE-226</t>
+          <t>CUE-173</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4294,19 +4294,19 @@
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Tray thud, tool clatter, mud squish, flag rope.</t>
+          <t>Rec hall foundation shake.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AST-069</t>
+          <t>AST-070</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Rumble / Building Shake</t>
+          <t>Running Footsteps</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4334,17 +4334,17 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/rumble_building_shake.wav</t>
+          <t>assets/sfx/running_footsteps.wav</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>6s</t>
+          <t>4s</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>CUE-173</t>
+          <t>CUE-012, CUE-204, CUE-132, CUE-144</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -4355,19 +4355,19 @@
       <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Rec hall foundation shake.</t>
+          <t>Chases, bunk exits, night runs.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AST-070</t>
+          <t>AST-072</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Running Footsteps</t>
+          <t>Slapstick Comedy Pack</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -4395,17 +4395,17 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/running_footsteps.wav</t>
+          <t>assets/sfx/slapstick_comedy_pack.wav</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>4s</t>
+          <t>1-3s</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>CUE-012, CUE-204, CUE-132, CUE-144</t>
+          <t>CUE-009, CUE-128, CUE-130</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
@@ -4416,19 +4416,19 @@
       <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Chases, bunk exits, night runs.</t>
+          <t>Rake bonk, banana slip, bucket clunk.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AST-072</t>
+          <t>AST-073</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Slapstick Comedy Pack</t>
+          <t>Smooch / Makeout</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4456,17 +4456,17 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/slapstick_comedy_pack.wav</t>
+          <t>assets/sfx/smooch_makeout.wav</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>1-3s</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>CUE-009, CUE-128, CUE-130</t>
+          <t>CUE-010, CUE-021, CUE-077</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -4477,24 +4477,24 @@
       <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Rake bonk, banana slip, bucket clunk.</t>
+          <t>Comedy smooch layers.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>AST-073</t>
+          <t>AST-075</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Smooch / Makeout</t>
+          <t>Scene Transition Whoosh</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>SFX</t>
+          <t>Transition</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/smooch_makeout.wav</t>
+          <t>assets/sfx/scene_transition_whoosh.wav</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>CUE-010, CUE-021, CUE-077</t>
+          <t>CUE-003, CUE-006, CUE-065, CUE-118, CUE-183, CUE-192</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -4538,33 +4538,33 @@
       <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Comedy smooch layers.</t>
+          <t>Cuts, dissolves, title cards, montage ticks.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>AST-075</t>
+          <t>AST-076</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Scene Transition Whoosh</t>
+          <t>VCR / Projector</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Transition</t>
+          <t>SFX</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4578,17 +4578,17 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/scene_transition_whoosh.wav</t>
+          <t>assets/sfx/vcr_projector_loop.wav</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>Loop</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>CUE-003, CUE-006, CUE-065, CUE-118, CUE-183, CUE-192</t>
+          <t>CUE-050, CUE-194</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -4599,19 +4599,19 @@
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Cuts, dissolves, title cards, montage ticks.</t>
+          <t>BetaMax gag + epilogue projector.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>AST-076</t>
+          <t>AST-077</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>VCR / Projector</t>
+          <t>Bus Diesel</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>One Shot</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4639,17 +4639,17 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vcr_projector_loop.wav</t>
+          <t>assets/sfx/vehicle_bus_diesel.wav</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Loop</t>
+          <t>6s</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>CUE-050, CUE-194</t>
+          <t>CUE-087, CUE-088</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -4660,19 +4660,19 @@
       <c r="L69" s="2" t="inlineStr"/>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>BetaMax gag + epilogue projector.</t>
+          <t>Tiger Claw arrival/departure.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>AST-077</t>
+          <t>AST-078</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Bus Diesel</t>
+          <t>Motorcycle</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4700,17 +4700,17 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vehicle_bus_diesel.wav</t>
+          <t>assets/sfx/vehicle_motorcycle.wav</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>6s</t>
+          <t>4s</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>CUE-087, CUE-088</t>
+          <t>CUE-079, CUE-080, CUE-082, CUE-136</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -4721,19 +4721,19 @@
       <c r="L70" s="2" t="inlineStr"/>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>Tiger Claw arrival/departure.</t>
+          <t>Approach, start, skid, night arrival.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>AST-078</t>
+          <t>AST-079</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Motorcycle</t>
+          <t>Truck / Pickup</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vehicle_motorcycle.wav</t>
+          <t>assets/sfx/vehicle_truck_pickup.wav</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>CUE-079, CUE-080, CUE-082, CUE-136</t>
+          <t>CUE-061, CUE-206</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
@@ -4782,19 +4782,19 @@
       <c r="L71" s="2" t="inlineStr"/>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Approach, start, skid, night arrival.</t>
+          <t>Beth's truck, door, peel-out.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>AST-079</t>
+          <t>AST-080</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Truck / Pickup</t>
+          <t>Van Engine</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vehicle_truck_pickup.wav</t>
+          <t>assets/sfx/vehicle_van_engine.wav</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>CUE-061, CUE-206</t>
+          <t>CUE-068</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4843,19 +4843,19 @@
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Beth's truck, door, peel-out.</t>
+          <t>Acceleration, doors, raft fall.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>AST-080</t>
+          <t>AST-081</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Van Engine</t>
+          <t>Vocal Callout</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -4878,22 +4878,22 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Freesound</t>
+          <t>Live table read</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vehicle_van_engine.wav</t>
+          <t>assets/sfx/vocal_callout.wav</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>4s</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>CUE-068</t>
+          <t>CUE-028</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4904,19 +4904,19 @@
       <c r="L73" s="2" t="inlineStr"/>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>Acceleration, doors, raft fall.</t>
+          <t>DINNER, CAPTURE THE FLAG, kitchen yell.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>AST-081</t>
+          <t>AST-082</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Vocal Callout</t>
+          <t>Water Splash</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4939,22 +4939,22 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Live table read</t>
+          <t>Freesound</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/vocal_callout.wav</t>
+          <t>assets/sfx/water_splash.wav</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>4s</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>CUE-028</t>
+          <t>CUE-055, CUE-100, CUE-129</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4965,19 +4965,19 @@
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>DINNER, CAPTURE THE FLAG, kitchen yell.</t>
+          <t>Lake fall, pool, ski drag.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>AST-082</t>
+          <t>AST-083</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Water Splash</t>
+          <t>Whistle</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -5005,17 +5005,17 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/water_splash.wav</t>
+          <t>assets/sfx/whistle.wav</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>4s</t>
+          <t>2s</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>CUE-055, CUE-100, CUE-129</t>
+          <t>CUE-054, CUE-093</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -5026,19 +5026,19 @@
       <c r="L75" s="2" t="inlineStr"/>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Lake fall, pool, ski drag.</t>
+          <t>Capture flag, wolf whistles.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>AST-083</t>
+          <t>AST-084</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Whistle</t>
+          <t>Wind Heavy / Gust</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -5066,17 +5066,17 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/whistle.wav</t>
+          <t>assets/sfx/wind_heavy_gust.wav</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>2s</t>
+          <t>15s</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>CUE-054, CUE-093</t>
+          <t>CUE-174, CUE-177</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
@@ -5087,19 +5087,19 @@
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Capture flag, wolf whistles.</t>
+          <t>Steve power + Skylab redirect gust.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>AST-084</t>
+          <t>AST-085</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Wind Heavy / Gust</t>
+          <t>Wind Gentle</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -5127,17 +5127,17 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/wind_heavy_gust.wav</t>
+          <t>assets/sfx/wind_gentle.wav</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>15s</t>
+          <t>3s</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>CUE-174, CUE-177</t>
+          <t>CUE-172</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -5148,33 +5148,33 @@
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Steve power + Skylab redirect gust.</t>
+          <t>Steve's initial breeze.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>AST-085</t>
+          <t>AST-086</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Wind Gentle</t>
+          <t>Silence Hold</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>SFX</t>
+          <t>Silence</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>One Shot</t>
+          <t>Silence</t>
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -5183,22 +5183,22 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Freesound</t>
+          <t>Digital silence</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>assets/sfx/wind_gentle.wav</t>
+          <t>assets/generated/silence_hold.mp3</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>3s</t>
+          <t>Variable</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
         <is>
-          <t>CUE-172</t>
+          <t>CUE-001, CUE-199, CUE-027, CUE-202, CUE-041, CUE-042, CUE-046, CUE-048, CUE-056, CUE-207, CUE-084, CUE-086, CUE-220, CUE-222, CUE-142, CUE-229, CUE-155, CUE-233, CUE-171, CUE-179, CUE-190</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -5208,67 +5208,6 @@
       </c>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr">
-        <is>
-          <t>Steve's initial breeze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>AST-086</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>Silence Hold</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>Silence</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>Silence</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t>Digital silence</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>assets/generated/silence_hold.mp3</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>CUE-001, CUE-199, CUE-027, CUE-202, CUE-041, CUE-042, CUE-046, CUE-048, CUE-056, CUE-207, CUE-084, CUE-086, CUE-220, CUE-222, CUE-142, CUE-229, CUE-155, CUE-233, CUE-171, CUE-179, CUE-190</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>Needed</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr"/>
-      <c r="M79" s="2" t="inlineStr">
         <is>
           <t>Reusable silence bed; cue duration/fade control behavior.</t>
         </is>

</xml_diff>